<commit_message>
updated merging cell counts to have the unpublished DosSantos 2020
</commit_message>
<xml_diff>
--- a/Young_etal_2013/Young_etal_2013.xlsx
+++ b/Young_etal_2013/Young_etal_2013.xlsx
@@ -2110,8 +2110,8 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d42a73f51a03135be35f4acb272f8cf1">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2ea21b36c10eaa86a5cb337ec7f4e0a6" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="335184889d0d2a5c2061d8ade3fa09f8">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2aa00a135f029e3b306b046578247198" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
     <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
     <xsd:element name="properties">
@@ -2384,22 +2384,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9574DCAA-0DC8-4FD9-B486-4FC4712ACA66}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{841B9D73-AB41-451B-BF9A-20C5178F8EF1}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>